<commit_message>
d1 (+4) on crouch
</commit_message>
<xml_diff>
--- a/data/azucena/inputs/azu_12bplus8_reina_v2.xlsx
+++ b/data/azucena/inputs/azu_12bplus8_reina_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dfa238\pyproj\gambit_tekken8\data\azucena\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D959D832-5B8C-487D-A873-BC9BFEE0707F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8032E375-6A87-4C5B-9F79-630A9840F8E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28740" yWindow="1125" windowWidth="28365" windowHeight="14355" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24225" yWindow="885" windowWidth="25620" windowHeight="14355" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
   <si>
     <t>key</t>
   </si>
@@ -117,6 +117,9 @@
   </si>
   <si>
     <t>d1</t>
+  </si>
+  <si>
+    <t>db1</t>
   </si>
 </sst>
 </file>
@@ -538,7 +541,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" customWidth="1"/>
@@ -964,7 +967,7 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -992,6 +995,38 @@
       </c>
       <c r="J14">
         <v>-43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15">
+        <v>5.2</v>
+      </c>
+      <c r="C15">
+        <v>20</v>
+      </c>
+      <c r="D15">
+        <v>-24</v>
+      </c>
+      <c r="E15">
+        <v>-6</v>
+      </c>
+      <c r="F15">
+        <v>20</v>
+      </c>
+      <c r="G15">
+        <v>20</v>
+      </c>
+      <c r="H15">
+        <v>-3</v>
+      </c>
+      <c r="I15">
+        <v>16</v>
+      </c>
+      <c r="J15">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>